<commit_message>
OK compound Testy + status in dashboard
</commit_message>
<xml_diff>
--- a/data/Testy.xlsx
+++ b/data/Testy.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="params" sheetId="1" state="visible" r:id="rId3"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
   <si>
     <t xml:space="preserve">name</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">timezon</t>
   </si>
   <si>
-    <t xml:space="preserve">Etc/GMT-12</t>
+    <t xml:space="preserve">Etc/GMT+12</t>
   </si>
   <si>
     <t xml:space="preserve">location</t>
@@ -84,6 +84,9 @@
     <t xml:space="preserve">container</t>
   </si>
   <si>
+    <t xml:space="preserve">after</t>
+  </si>
+  <si>
     <t xml:space="preserve">delete</t>
   </si>
   <si>
@@ -94,6 +97,18 @@
   </si>
   <si>
     <t xml:space="preserve">Children / teens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">insert1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service d0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Service after d0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fillin</t>
   </si>
 </sst>
 </file>
@@ -431,7 +446,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -444,39 +459,83 @@
       <c r="C1" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="D1" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="D2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>22</v>
-      </c>
+      <c r="D3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D8" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>